<commit_message>
#18 LCD connector changed back to the existing one
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_MCM_v1.6/BOM/Client-BOM-OFP_MCM_v1.6.xlsx
+++ b/Design-Files/OFP_MCM_v1.6/BOM/Client-BOM-OFP_MCM_v1.6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\nabilfesal-smartmeter-hw\Design-Files\OFP_MCM_v1.6\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A98945-5294-4151-BCE5-7C6D46AA9351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{921413CF-EB97-46D2-9211-A9537C381431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -615,12 +615,6 @@
     <t>J4</t>
   </si>
   <si>
-    <t>CONN FFC BOTTOM 40POS 0.5MM R/A</t>
-  </si>
-  <si>
-    <t>FH41-40S-0.5SH(05)</t>
-  </si>
-  <si>
     <t>Hirose</t>
   </si>
   <si>
@@ -1840,6 +1834,12 @@
   </si>
   <si>
     <t>SMF3.3</t>
+  </si>
+  <si>
+    <t>CONN FFC FPC 40POS 0.5MM R/A Top Bottom</t>
+  </si>
+  <si>
+    <t>FH34SRJ-40S-0.5SH(50)</t>
   </si>
 </sst>
 </file>
@@ -3663,16 +3663,16 @@
         <v>168</v>
       </c>
       <c r="D40" s="9" t="s">
+        <v>597</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="F40" s="9" t="s">
         <v>599</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="G40" s="10" t="s">
         <v>600</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>601</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>602</v>
       </c>
       <c r="H40" s="9" t="s">
         <v>172</v>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="K44" s="9"/>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" spans="1:11" ht="24">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
         <f t="shared" si="1"/>
@@ -3826,16 +3826,16 @@
         <v>193</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>194</v>
+        <v>601</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>195</v>
+        <v>602</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I45" s="10" t="s">
         <v>145</v>
@@ -3852,22 +3852,22 @@
         <v>44</v>
       </c>
       <c r="C46" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>197</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>199</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I46" s="10" t="s">
         <v>145</v>
@@ -3884,22 +3884,22 @@
         <v>45</v>
       </c>
       <c r="C47" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="E47" s="15" t="s">
         <v>197</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>201</v>
-      </c>
-      <c r="E47" s="15" t="s">
-        <v>199</v>
       </c>
       <c r="F47" s="14" t="s">
         <v>34</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I47" s="15" t="s">
         <v>136</v>
@@ -3918,22 +3918,22 @@
         <v>46</v>
       </c>
       <c r="C48" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>202</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>204</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="I48" s="10" t="s">
         <v>145</v>
@@ -3950,25 +3950,25 @@
         <v>47</v>
       </c>
       <c r="C49" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>209</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G49" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="H49" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="I49" s="10" t="s">
         <v>210</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="I49" s="10" t="s">
-        <v>212</v>
       </c>
       <c r="J49" s="9">
         <v>1</v>
@@ -3982,25 +3982,25 @@
         <v>48</v>
       </c>
       <c r="C50" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E50" s="13" t="s">
         <v>213</v>
-      </c>
-      <c r="D50" s="12" t="s">
-        <v>214</v>
-      </c>
-      <c r="E50" s="13" t="s">
-        <v>215</v>
       </c>
       <c r="F50" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G50" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I50" s="13" t="s">
         <v>216</v>
-      </c>
-      <c r="H50" s="12" t="s">
-        <v>217</v>
-      </c>
-      <c r="I50" s="13" t="s">
-        <v>218</v>
       </c>
       <c r="J50" s="12">
         <v>3</v>
@@ -4014,25 +4014,25 @@
         <v>49</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G51" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="J51" s="9">
         <v>1</v>
@@ -4046,25 +4046,25 @@
         <v>50</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G52" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="H52" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="I52" s="13" t="s">
         <v>225</v>
-      </c>
-      <c r="H52" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="I52" s="13" t="s">
-        <v>227</v>
       </c>
       <c r="J52" s="12">
         <v>1</v>
@@ -4078,19 +4078,19 @@
         <v>51</v>
       </c>
       <c r="C53" s="11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>176</v>
       </c>
       <c r="G53" s="15" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H53" s="14" t="s">
         <v>15</v>
@@ -4112,22 +4112,22 @@
         <v>52</v>
       </c>
       <c r="C54" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="E54" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="D54" s="12" t="s">
+      <c r="F54" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="E54" s="13" t="s">
+      <c r="G54" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="F54" s="12" t="s">
+      <c r="H54" s="12" t="s">
         <v>234</v>
-      </c>
-      <c r="G54" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="H54" s="12" t="s">
-        <v>236</v>
       </c>
       <c r="I54" s="13" t="s">
         <v>145</v>
@@ -4144,22 +4144,22 @@
         <v>53</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D55" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="F55" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="G55" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="H55" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="G55" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>241</v>
       </c>
       <c r="I55" s="13" t="s">
         <v>145</v>
@@ -4176,22 +4176,22 @@
         <v>54</v>
       </c>
       <c r="C56" s="11" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D56" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="F56" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="E56" s="13" t="s">
+      <c r="G56" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="F56" s="12" t="s">
+      <c r="H56" s="12" t="s">
         <v>244</v>
-      </c>
-      <c r="G56" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="H56" s="12" t="s">
-        <v>246</v>
       </c>
       <c r="I56" s="13" t="s">
         <v>145</v>
@@ -4208,22 +4208,22 @@
         <v>55</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="F57" s="9" t="s">
         <v>247</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="G57" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="F57" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="G57" s="10" t="s">
-        <v>250</v>
-      </c>
       <c r="H57" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="I57" s="13" t="s">
         <v>145</v>
@@ -4240,22 +4240,22 @@
         <v>56</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D58" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="F58" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="G58" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="E58" s="13" t="s">
-        <v>252</v>
-      </c>
-      <c r="F58" s="12" t="s">
+      <c r="H58" s="12" t="s">
         <v>239</v>
-      </c>
-      <c r="G58" s="13" t="s">
-        <v>253</v>
-      </c>
-      <c r="H58" s="12" t="s">
-        <v>241</v>
       </c>
       <c r="I58" s="13" t="s">
         <v>145</v>
@@ -4272,22 +4272,22 @@
         <v>57</v>
       </c>
       <c r="C59" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="E59" s="10" t="s">
         <v>254</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>256</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G59" s="10" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="I59" s="13" t="s">
         <v>145</v>
@@ -4304,19 +4304,19 @@
         <v>58</v>
       </c>
       <c r="C60" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="E60" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="D60" s="12" t="s">
+      <c r="F60" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="E60" s="13" t="s">
+      <c r="G60" s="13" t="s">
         <v>261</v>
-      </c>
-      <c r="F60" s="12" t="s">
-        <v>262</v>
-      </c>
-      <c r="G60" s="13" t="s">
-        <v>263</v>
       </c>
       <c r="H60" s="12" t="s">
         <v>156</v>
@@ -4336,22 +4336,22 @@
         <v>59</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D61" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="F61" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="E61" s="10" t="s">
+      <c r="G61" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="F61" s="9" t="s">
+      <c r="H61" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="G61" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>268</v>
       </c>
       <c r="I61" s="13" t="s">
         <v>145</v>
@@ -4368,25 +4368,25 @@
         <v>60</v>
       </c>
       <c r="C62" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="E62" s="13" t="s">
         <v>269</v>
       </c>
-      <c r="D62" s="12" t="s">
+      <c r="F62" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="E62" s="13" t="s">
+      <c r="G62" s="13" t="s">
         <v>271</v>
-      </c>
-      <c r="F62" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G62" s="13" t="s">
-        <v>273</v>
       </c>
       <c r="H62" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I62" s="13" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="J62" s="12">
         <v>7</v>
@@ -4400,25 +4400,25 @@
         <v>61</v>
       </c>
       <c r="C63" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D63" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G63" s="10" t="s">
         <v>275</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="F63" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G63" s="10" t="s">
-        <v>277</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="J63" s="9">
         <v>1</v>
@@ -4432,25 +4432,25 @@
         <v>62</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D64" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="F64" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G64" s="13" t="s">
         <v>279</v>
-      </c>
-      <c r="E64" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="F64" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G64" s="13" t="s">
-        <v>281</v>
       </c>
       <c r="H64" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I64" s="13" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J64" s="12">
         <v>1</v>
@@ -4464,25 +4464,25 @@
         <v>63</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D65" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="F65" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G65" s="10" t="s">
         <v>283</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>284</v>
-      </c>
-      <c r="F65" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G65" s="10" t="s">
-        <v>285</v>
       </c>
       <c r="H65" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I65" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J65" s="9">
         <v>1</v>
@@ -4496,25 +4496,25 @@
         <v>64</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D66" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="F66" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G66" s="13" t="s">
         <v>287</v>
-      </c>
-      <c r="E66" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="F66" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G66" s="13" t="s">
-        <v>289</v>
       </c>
       <c r="H66" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I66" s="13" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J66" s="12">
         <v>1</v>
@@ -4528,25 +4528,25 @@
         <v>65</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D67" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="E67" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F67" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="G67" s="10" t="s">
         <v>292</v>
-      </c>
-      <c r="F67" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G67" s="10" t="s">
-        <v>294</v>
       </c>
       <c r="H67" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I67" s="10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J67" s="9">
         <v>1</v>
@@ -4560,25 +4560,25 @@
         <v>66</v>
       </c>
       <c r="C68" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="E68" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="D68" s="12" t="s">
+      <c r="F68" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G68" s="13" t="s">
         <v>297</v>
-      </c>
-      <c r="E68" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="F68" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G68" s="13" t="s">
-        <v>299</v>
       </c>
       <c r="H68" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I68" s="13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J68" s="12">
         <v>1</v>
@@ -4592,25 +4592,25 @@
         <v>67</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D69" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="E69" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="F69" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G69" s="10" t="s">
         <v>301</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="F69" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G69" s="10" t="s">
-        <v>303</v>
       </c>
       <c r="H69" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I69" s="10" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J69" s="9">
         <v>1</v>
@@ -4624,25 +4624,25 @@
         <v>68</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D70" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="E70" s="13" t="s">
+        <v>304</v>
+      </c>
+      <c r="F70" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G70" s="13" t="s">
         <v>305</v>
-      </c>
-      <c r="E70" s="13" t="s">
-        <v>306</v>
-      </c>
-      <c r="F70" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G70" s="13" t="s">
-        <v>307</v>
       </c>
       <c r="H70" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I70" s="13" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J70" s="12">
         <v>1</v>
@@ -4656,25 +4656,25 @@
         <v>69</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D71" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="E71" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G71" s="10" t="s">
         <v>308</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>309</v>
-      </c>
-      <c r="F71" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G71" s="10" t="s">
-        <v>310</v>
       </c>
       <c r="H71" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I71" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J71" s="9">
         <v>1</v>
@@ -4688,25 +4688,25 @@
         <v>70</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D72" s="12" t="s">
+        <v>310</v>
+      </c>
+      <c r="E72" s="13" t="s">
+        <v>311</v>
+      </c>
+      <c r="F72" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G72" s="13" t="s">
         <v>312</v>
-      </c>
-      <c r="E72" s="13" t="s">
-        <v>313</v>
-      </c>
-      <c r="F72" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G72" s="13" t="s">
-        <v>314</v>
       </c>
       <c r="H72" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I72" s="13" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J72" s="12">
         <v>1</v>
@@ -4720,25 +4720,25 @@
         <v>71</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D73" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="E73" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G73" s="10" t="s">
         <v>316</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>317</v>
-      </c>
-      <c r="F73" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G73" s="10" t="s">
-        <v>318</v>
       </c>
       <c r="H73" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I73" s="10" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J73" s="9">
         <v>6</v>
@@ -4752,25 +4752,25 @@
         <v>72</v>
       </c>
       <c r="C74" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D74" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="E74" s="13" t="s">
+        <v>319</v>
+      </c>
+      <c r="F74" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G74" s="13" t="s">
         <v>320</v>
-      </c>
-      <c r="E74" s="13" t="s">
-        <v>321</v>
-      </c>
-      <c r="F74" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G74" s="13" t="s">
-        <v>322</v>
       </c>
       <c r="H74" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I74" s="13" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J74" s="12">
         <v>1</v>
@@ -4784,25 +4784,25 @@
         <v>73</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D75" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G75" s="10" t="s">
         <v>324</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>325</v>
-      </c>
-      <c r="F75" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G75" s="10" t="s">
-        <v>326</v>
       </c>
       <c r="H75" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I75" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J75" s="9">
         <v>18</v>
@@ -4816,25 +4816,25 @@
         <v>74</v>
       </c>
       <c r="C76" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D76" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="E76" s="13" t="s">
+        <v>327</v>
+      </c>
+      <c r="F76" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G76" s="13" t="s">
         <v>328</v>
-      </c>
-      <c r="E76" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="F76" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G76" s="13" t="s">
-        <v>330</v>
       </c>
       <c r="H76" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I76" s="13" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J76" s="12">
         <v>2</v>
@@ -4848,25 +4848,25 @@
         <v>75</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D77" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="E77" s="10" t="s">
+        <v>331</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G77" s="10" t="s">
         <v>332</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="F77" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G77" s="10" t="s">
-        <v>334</v>
       </c>
       <c r="H77" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J77" s="9">
         <v>1</v>
@@ -4880,25 +4880,25 @@
         <v>76</v>
       </c>
       <c r="C78" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D78" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="E78" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="F78" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G78" s="13" t="s">
         <v>336</v>
-      </c>
-      <c r="E78" s="13" t="s">
-        <v>337</v>
-      </c>
-      <c r="F78" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G78" s="13" t="s">
-        <v>338</v>
       </c>
       <c r="H78" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I78" s="13" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J78" s="12">
         <v>1</v>
@@ -4912,25 +4912,25 @@
         <v>77</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D79" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="E79" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G79" s="10" t="s">
         <v>340</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="F79" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G79" s="10" t="s">
-        <v>342</v>
       </c>
       <c r="H79" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I79" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J79" s="9">
         <v>10</v>
@@ -4944,25 +4944,25 @@
         <v>78</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D80" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="E80" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="F80" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G80" s="13" t="s">
         <v>343</v>
-      </c>
-      <c r="E80" s="13" t="s">
-        <v>344</v>
-      </c>
-      <c r="F80" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G80" s="13" t="s">
-        <v>345</v>
       </c>
       <c r="H80" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I80" s="13" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="J80" s="12">
         <v>1</v>
@@ -4976,25 +4976,25 @@
         <v>79</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D81" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E81" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="F81" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G81" s="10" t="s">
         <v>347</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>348</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G81" s="10" t="s">
-        <v>349</v>
       </c>
       <c r="H81" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I81" s="10" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="J81" s="9">
         <v>1</v>
@@ -5008,25 +5008,25 @@
         <v>80</v>
       </c>
       <c r="C82" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D82" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="E82" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="F82" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G82" s="13" t="s">
         <v>351</v>
-      </c>
-      <c r="E82" s="13" t="s">
-        <v>352</v>
-      </c>
-      <c r="F82" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G82" s="13" t="s">
-        <v>353</v>
       </c>
       <c r="H82" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I82" s="13" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="J82" s="12">
         <v>1</v>
@@ -5040,25 +5040,25 @@
         <v>81</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D83" s="9" t="s">
+        <v>353</v>
+      </c>
+      <c r="E83" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="F83" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G83" s="10" t="s">
         <v>355</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>356</v>
-      </c>
-      <c r="F83" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G83" s="10" t="s">
-        <v>357</v>
       </c>
       <c r="H83" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I83" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J83" s="9">
         <v>1</v>
@@ -5072,25 +5072,25 @@
         <v>82</v>
       </c>
       <c r="C84" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D84" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="E84" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="F84" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G84" s="13" t="s">
         <v>359</v>
-      </c>
-      <c r="E84" s="13" t="s">
-        <v>360</v>
-      </c>
-      <c r="F84" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G84" s="13" t="s">
-        <v>361</v>
       </c>
       <c r="H84" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I84" s="13" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="J84" s="12">
         <v>1</v>
@@ -5104,25 +5104,25 @@
         <v>83</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D85" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="E85" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G85" s="10" t="s">
         <v>363</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>364</v>
-      </c>
-      <c r="F85" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G85" s="10" t="s">
-        <v>365</v>
       </c>
       <c r="H85" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J85" s="9">
         <v>7</v>
@@ -5136,25 +5136,25 @@
         <v>84</v>
       </c>
       <c r="C86" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D86" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="E86" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="F86" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G86" s="13" t="s">
         <v>366</v>
-      </c>
-      <c r="E86" s="13" t="s">
-        <v>367</v>
-      </c>
-      <c r="F86" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G86" s="13" t="s">
-        <v>368</v>
       </c>
       <c r="H86" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I86" s="13" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="J86" s="12">
         <v>4</v>
@@ -5168,25 +5168,25 @@
         <v>85</v>
       </c>
       <c r="C87" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D87" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E87" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G87" s="10" t="s">
         <v>370</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>371</v>
-      </c>
-      <c r="F87" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G87" s="10" t="s">
-        <v>372</v>
       </c>
       <c r="H87" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I87" s="10" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J87" s="9">
         <v>5</v>
@@ -5200,25 +5200,25 @@
         <v>86</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D88" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="E88" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="F88" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G88" s="13" t="s">
         <v>373</v>
-      </c>
-      <c r="E88" s="13" t="s">
-        <v>374</v>
-      </c>
-      <c r="F88" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G88" s="13" t="s">
-        <v>375</v>
       </c>
       <c r="H88" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I88" s="13" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="J88" s="12">
         <v>1</v>
@@ -5232,25 +5232,25 @@
         <v>87</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D89" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="E89" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="F89" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G89" s="17" t="s">
         <v>377</v>
-      </c>
-      <c r="E89" s="10" t="s">
-        <v>378</v>
-      </c>
-      <c r="F89" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G89" s="17" t="s">
-        <v>379</v>
       </c>
       <c r="H89" s="18" t="s">
         <v>74</v>
       </c>
       <c r="I89" s="10" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="J89" s="9">
         <v>2</v>
@@ -5264,25 +5264,25 @@
         <v>88</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D90" s="12" t="s">
+        <v>379</v>
+      </c>
+      <c r="E90" s="13" t="s">
+        <v>380</v>
+      </c>
+      <c r="F90" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G90" s="13" t="s">
         <v>381</v>
-      </c>
-      <c r="E90" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="F90" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G90" s="13" t="s">
-        <v>383</v>
       </c>
       <c r="H90" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I90" s="13" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="J90" s="12">
         <v>1</v>
@@ -5296,25 +5296,25 @@
         <v>89</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D91" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="E91" s="10" t="s">
+        <v>384</v>
+      </c>
+      <c r="F91" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G91" s="10" t="s">
         <v>385</v>
-      </c>
-      <c r="E91" s="10" t="s">
-        <v>386</v>
-      </c>
-      <c r="F91" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G91" s="10" t="s">
-        <v>387</v>
       </c>
       <c r="H91" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I91" s="10" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="J91" s="9">
         <v>1</v>
@@ -5328,25 +5328,25 @@
         <v>90</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D92" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="E92" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="F92" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G92" s="13" t="s">
         <v>389</v>
-      </c>
-      <c r="E92" s="13" t="s">
-        <v>390</v>
-      </c>
-      <c r="F92" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G92" s="13" t="s">
-        <v>391</v>
       </c>
       <c r="H92" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I92" s="13" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="J92" s="12">
         <v>1</v>
@@ -5360,25 +5360,25 @@
         <v>91</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D93" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="E93" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="F93" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G93" s="10" t="s">
         <v>393</v>
-      </c>
-      <c r="E93" s="10" t="s">
-        <v>394</v>
-      </c>
-      <c r="F93" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G93" s="10" t="s">
-        <v>395</v>
       </c>
       <c r="H93" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I93" s="10" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="J93" s="9">
         <v>1</v>
@@ -5392,25 +5392,25 @@
         <v>92</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D94" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="E94" s="13" t="s">
+        <v>396</v>
+      </c>
+      <c r="F94" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G94" s="13" t="s">
         <v>397</v>
-      </c>
-      <c r="E94" s="13" t="s">
-        <v>398</v>
-      </c>
-      <c r="F94" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G94" s="13" t="s">
-        <v>399</v>
       </c>
       <c r="H94" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I94" s="13" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="J94" s="12">
         <v>1</v>
@@ -5424,25 +5424,25 @@
         <v>93</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D95" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="E95" s="10" t="s">
+        <v>400</v>
+      </c>
+      <c r="F95" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G95" s="10" t="s">
         <v>401</v>
-      </c>
-      <c r="E95" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="F95" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G95" s="10" t="s">
-        <v>403</v>
       </c>
       <c r="H95" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I95" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="J95" s="9">
         <v>1</v>
@@ -5456,25 +5456,25 @@
         <v>94</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D96" s="12" t="s">
+        <v>403</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G96" s="13" t="s">
         <v>405</v>
-      </c>
-      <c r="E96" s="13" t="s">
-        <v>406</v>
-      </c>
-      <c r="F96" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G96" s="13" t="s">
-        <v>407</v>
       </c>
       <c r="H96" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I96" s="13" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="J96" s="12">
         <v>3</v>
@@ -5488,25 +5488,25 @@
         <v>95</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D97" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="E97" s="10" t="s">
+        <v>408</v>
+      </c>
+      <c r="F97" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G97" s="10" t="s">
         <v>409</v>
-      </c>
-      <c r="E97" s="10" t="s">
-        <v>410</v>
-      </c>
-      <c r="F97" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G97" s="10" t="s">
-        <v>411</v>
       </c>
       <c r="H97" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I97" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="J97" s="9">
         <v>6</v>
@@ -5520,25 +5520,25 @@
         <v>96</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D98" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="E98" s="13" t="s">
+        <v>412</v>
+      </c>
+      <c r="F98" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G98" s="13" t="s">
         <v>413</v>
-      </c>
-      <c r="E98" s="13" t="s">
-        <v>414</v>
-      </c>
-      <c r="F98" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G98" s="13" t="s">
-        <v>415</v>
       </c>
       <c r="H98" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I98" s="13" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="J98" s="12">
         <v>1</v>
@@ -5552,25 +5552,25 @@
         <v>97</v>
       </c>
       <c r="C99" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D99" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E99" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G99" s="10" t="s">
         <v>417</v>
-      </c>
-      <c r="E99" s="10" t="s">
-        <v>418</v>
-      </c>
-      <c r="F99" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G99" s="10" t="s">
-        <v>419</v>
       </c>
       <c r="H99" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I99" s="10" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="J99" s="9">
         <v>1</v>
@@ -5584,25 +5584,25 @@
         <v>98</v>
       </c>
       <c r="C100" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D100" s="12" t="s">
+        <v>419</v>
+      </c>
+      <c r="E100" s="13" t="s">
+        <v>420</v>
+      </c>
+      <c r="F100" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G100" s="13" t="s">
         <v>421</v>
-      </c>
-      <c r="E100" s="13" t="s">
-        <v>422</v>
-      </c>
-      <c r="F100" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G100" s="13" t="s">
-        <v>423</v>
       </c>
       <c r="H100" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I100" s="13" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="J100" s="12">
         <v>1</v>
@@ -5616,25 +5616,25 @@
         <v>99</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D101" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="E101" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="F101" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G101" s="10" t="s">
         <v>425</v>
-      </c>
-      <c r="E101" s="10" t="s">
-        <v>426</v>
-      </c>
-      <c r="F101" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G101" s="10" t="s">
-        <v>427</v>
       </c>
       <c r="H101" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I101" s="10" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="J101" s="9">
         <v>2</v>
@@ -5648,19 +5648,19 @@
         <v>100</v>
       </c>
       <c r="C102" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D102" s="14" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E102" s="15" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="F102" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G102" s="15" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H102" s="14" t="s">
         <v>74</v>
@@ -5682,19 +5682,19 @@
         <v>101</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D103" s="14" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E103" s="15" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F103" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G103" s="15" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H103" s="14" t="s">
         <v>74</v>
@@ -5716,25 +5716,25 @@
         <v>102</v>
       </c>
       <c r="C104" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D104" s="12" t="s">
+        <v>429</v>
+      </c>
+      <c r="E104" s="13" t="s">
+        <v>430</v>
+      </c>
+      <c r="F104" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="G104" s="13" t="s">
         <v>431</v>
-      </c>
-      <c r="E104" s="13" t="s">
-        <v>432</v>
-      </c>
-      <c r="F104" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="G104" s="13" t="s">
-        <v>433</v>
       </c>
       <c r="H104" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I104" s="13" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="J104" s="12">
         <v>1</v>
@@ -5748,25 +5748,25 @@
         <v>103</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D105" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="E105" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="F105" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G105" s="10" t="s">
         <v>435</v>
-      </c>
-      <c r="E105" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="F105" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G105" s="10" t="s">
-        <v>437</v>
       </c>
       <c r="H105" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I105" s="10" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="J105" s="9">
         <v>1</v>
@@ -5780,25 +5780,25 @@
         <v>104</v>
       </c>
       <c r="C106" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D106" s="12" t="s">
+        <v>437</v>
+      </c>
+      <c r="E106" s="13" t="s">
+        <v>438</v>
+      </c>
+      <c r="F106" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G106" s="13" t="s">
         <v>439</v>
-      </c>
-      <c r="E106" s="13" t="s">
-        <v>440</v>
-      </c>
-      <c r="F106" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G106" s="13" t="s">
-        <v>441</v>
       </c>
       <c r="H106" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I106" s="13" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="J106" s="12">
         <v>1</v>
@@ -5812,25 +5812,25 @@
         <v>105</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D107" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="E107" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="F107" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G107" s="10" t="s">
         <v>443</v>
-      </c>
-      <c r="E107" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="F107" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G107" s="10" t="s">
-        <v>445</v>
       </c>
       <c r="H107" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I107" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J107" s="9">
         <v>1</v>
@@ -5844,19 +5844,19 @@
         <v>106</v>
       </c>
       <c r="C108" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D108" s="14" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="E108" s="15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="F108" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G108" s="15" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="H108" s="14" t="s">
         <v>74</v>
@@ -5878,25 +5878,25 @@
         <v>107</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D109" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E109" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="F109" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G109" s="10" t="s">
         <v>447</v>
-      </c>
-      <c r="E109" s="10" t="s">
-        <v>448</v>
-      </c>
-      <c r="F109" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G109" s="10" t="s">
-        <v>449</v>
       </c>
       <c r="H109" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I109" s="10" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="J109" s="9">
         <v>1</v>
@@ -5910,19 +5910,19 @@
         <v>108</v>
       </c>
       <c r="C110" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D110" s="14" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="E110" s="15" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="F110" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G110" s="15" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="H110" s="14" t="s">
         <v>74</v>
@@ -5944,25 +5944,25 @@
         <v>109</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D111" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="E111" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="F111" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="G111" s="10" t="s">
         <v>451</v>
-      </c>
-      <c r="E111" s="10" t="s">
-        <v>452</v>
-      </c>
-      <c r="F111" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="G111" s="10" t="s">
-        <v>453</v>
       </c>
       <c r="H111" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I111" s="10" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="J111" s="9">
         <v>4</v>
@@ -5976,25 +5976,25 @@
         <v>110</v>
       </c>
       <c r="C112" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D112" s="12" t="s">
+        <v>453</v>
+      </c>
+      <c r="E112" s="13" t="s">
+        <v>454</v>
+      </c>
+      <c r="F112" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="G112" s="13" t="s">
         <v>455</v>
-      </c>
-      <c r="E112" s="13" t="s">
-        <v>456</v>
-      </c>
-      <c r="F112" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="G112" s="13" t="s">
-        <v>457</v>
       </c>
       <c r="H112" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I112" s="13" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J112" s="12">
         <v>1</v>
@@ -6008,19 +6008,19 @@
         <v>111</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D113" s="14" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E113" s="15" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="F113" s="14" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G113" s="15" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="H113" s="14" t="s">
         <v>74</v>
@@ -6042,19 +6042,19 @@
         <v>112</v>
       </c>
       <c r="C114" s="11" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D114" s="14" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="E114" s="15" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="F114" s="14" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G114" s="15" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H114" s="14" t="s">
         <v>74</v>
@@ -6076,25 +6076,25 @@
         <v>113</v>
       </c>
       <c r="C115" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D115" s="12" t="s">
+        <v>458</v>
+      </c>
+      <c r="E115" s="13" t="s">
+        <v>459</v>
+      </c>
+      <c r="F115" s="12" t="s">
         <v>460</v>
       </c>
-      <c r="E115" s="13" t="s">
+      <c r="G115" s="13" t="s">
         <v>461</v>
-      </c>
-      <c r="F115" s="12" t="s">
-        <v>462</v>
-      </c>
-      <c r="G115" s="13" t="s">
-        <v>463</v>
       </c>
       <c r="H115" s="12" t="s">
         <v>74</v>
       </c>
       <c r="I115" s="13" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="J115" s="12">
         <v>6</v>
@@ -6108,25 +6108,25 @@
         <v>114</v>
       </c>
       <c r="C116" s="11" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D116" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="E116" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="F116" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G116" s="10" t="s">
         <v>464</v>
-      </c>
-      <c r="E116" s="10" t="s">
-        <v>465</v>
-      </c>
-      <c r="F116" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="G116" s="10" t="s">
-        <v>466</v>
       </c>
       <c r="H116" s="9" t="s">
         <v>74</v>
       </c>
       <c r="I116" s="10" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="J116" s="9">
         <v>1</v>
@@ -6140,22 +6140,22 @@
         <v>115</v>
       </c>
       <c r="C117" s="11" t="s">
+        <v>466</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>467</v>
+      </c>
+      <c r="E117" s="13" t="s">
         <v>468</v>
-      </c>
-      <c r="D117" s="12" t="s">
-        <v>469</v>
-      </c>
-      <c r="E117" s="13" t="s">
-        <v>470</v>
       </c>
       <c r="F117" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G117" s="13" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="H117" s="12" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="I117" s="13" t="s">
         <v>145</v>
@@ -6172,22 +6172,22 @@
         <v>116</v>
       </c>
       <c r="C118" s="8" t="s">
+        <v>471</v>
+      </c>
+      <c r="D118" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="E118" s="10" t="s">
         <v>473</v>
-      </c>
-      <c r="D118" s="9" t="s">
-        <v>474</v>
-      </c>
-      <c r="E118" s="10" t="s">
-        <v>475</v>
       </c>
       <c r="F118" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G118" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="H118" s="9" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="I118" s="13" t="s">
         <v>145</v>
@@ -6204,22 +6204,22 @@
         <v>117</v>
       </c>
       <c r="C119" s="11" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="D119" s="12" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="F119" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G119" s="13" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="H119" s="12" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="I119" s="13" t="s">
         <v>145</v>
@@ -6236,22 +6236,22 @@
         <v>118</v>
       </c>
       <c r="C120" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="D120" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="E120" s="10" t="s">
         <v>481</v>
       </c>
-      <c r="D120" s="9" t="s">
+      <c r="F120" s="9" t="s">
         <v>482</v>
       </c>
-      <c r="E120" s="10" t="s">
+      <c r="G120" s="10" t="s">
         <v>483</v>
       </c>
-      <c r="F120" s="9" t="s">
+      <c r="H120" s="9" t="s">
         <v>484</v>
-      </c>
-      <c r="G120" s="10" t="s">
-        <v>485</v>
-      </c>
-      <c r="H120" s="9" t="s">
-        <v>486</v>
       </c>
       <c r="I120" s="13" t="s">
         <v>145</v>
@@ -6268,22 +6268,22 @@
         <v>119</v>
       </c>
       <c r="C121" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D121" s="12" t="s">
+        <v>485</v>
+      </c>
+      <c r="E121" s="13" t="s">
+        <v>486</v>
+      </c>
+      <c r="F121" s="12" t="s">
         <v>487</v>
       </c>
-      <c r="E121" s="13" t="s">
+      <c r="G121" s="13" t="s">
         <v>488</v>
       </c>
-      <c r="F121" s="12" t="s">
+      <c r="H121" s="12" t="s">
         <v>489</v>
-      </c>
-      <c r="G121" s="13" t="s">
-        <v>490</v>
-      </c>
-      <c r="H121" s="12" t="s">
-        <v>491</v>
       </c>
       <c r="I121" s="13" t="s">
         <v>145</v>
@@ -6300,22 +6300,22 @@
         <v>120</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D122" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="E122" s="10" t="s">
+        <v>491</v>
+      </c>
+      <c r="F122" s="9" t="s">
         <v>492</v>
       </c>
-      <c r="E122" s="10" t="s">
+      <c r="G122" s="10" t="s">
         <v>493</v>
       </c>
-      <c r="F122" s="9" t="s">
+      <c r="H122" s="9" t="s">
         <v>494</v>
-      </c>
-      <c r="G122" s="10" t="s">
-        <v>495</v>
-      </c>
-      <c r="H122" s="9" t="s">
-        <v>496</v>
       </c>
       <c r="I122" s="13" t="s">
         <v>145</v>
@@ -6332,22 +6332,22 @@
         <v>121</v>
       </c>
       <c r="C123" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D123" s="12" t="s">
+        <v>495</v>
+      </c>
+      <c r="E123" s="13" t="s">
+        <v>496</v>
+      </c>
+      <c r="F123" s="12" t="s">
         <v>497</v>
       </c>
-      <c r="E123" s="13" t="s">
+      <c r="G123" s="13" t="s">
         <v>498</v>
       </c>
-      <c r="F123" s="12" t="s">
+      <c r="H123" s="12" t="s">
         <v>499</v>
-      </c>
-      <c r="G123" s="13" t="s">
-        <v>500</v>
-      </c>
-      <c r="H123" s="12" t="s">
-        <v>501</v>
       </c>
       <c r="I123" s="13" t="s">
         <v>145</v>
@@ -6364,22 +6364,22 @@
         <v>122</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D124" s="9" t="s">
+        <v>500</v>
+      </c>
+      <c r="E124" s="10" t="s">
+        <v>501</v>
+      </c>
+      <c r="F124" s="9" t="s">
         <v>502</v>
       </c>
-      <c r="E124" s="10" t="s">
+      <c r="G124" s="10" t="s">
         <v>503</v>
       </c>
-      <c r="F124" s="9" t="s">
+      <c r="H124" s="9" t="s">
         <v>504</v>
-      </c>
-      <c r="G124" s="10" t="s">
-        <v>505</v>
-      </c>
-      <c r="H124" s="9" t="s">
-        <v>506</v>
       </c>
       <c r="I124" s="13" t="s">
         <v>145</v>
@@ -6396,22 +6396,22 @@
         <v>123</v>
       </c>
       <c r="C125" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D125" s="12" t="s">
+        <v>505</v>
+      </c>
+      <c r="E125" s="13" t="s">
+        <v>506</v>
+      </c>
+      <c r="F125" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="E125" s="13" t="s">
+      <c r="G125" s="13" t="s">
         <v>508</v>
       </c>
-      <c r="F125" s="12" t="s">
-        <v>509</v>
-      </c>
-      <c r="G125" s="13" t="s">
-        <v>510</v>
-      </c>
       <c r="H125" s="12" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I125" s="13" t="s">
         <v>145</v>
@@ -6428,22 +6428,22 @@
         <v>124</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D126" s="9" t="s">
+        <v>509</v>
+      </c>
+      <c r="E126" s="10" t="s">
+        <v>510</v>
+      </c>
+      <c r="F126" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="E126" s="10" t="s">
+      <c r="G126" s="10" t="s">
         <v>512</v>
       </c>
-      <c r="F126" s="9" t="s">
-        <v>513</v>
-      </c>
-      <c r="G126" s="10" t="s">
-        <v>514</v>
-      </c>
       <c r="H126" s="9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I126" s="13" t="s">
         <v>145</v>
@@ -6460,22 +6460,22 @@
         <v>125</v>
       </c>
       <c r="C127" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D127" s="12" t="s">
+        <v>513</v>
+      </c>
+      <c r="E127" s="13" t="s">
+        <v>514</v>
+      </c>
+      <c r="F127" s="12" t="s">
         <v>515</v>
       </c>
-      <c r="E127" s="13" t="s">
+      <c r="G127" s="13" t="s">
         <v>516</v>
       </c>
-      <c r="F127" s="12" t="s">
-        <v>517</v>
-      </c>
-      <c r="G127" s="13" t="s">
-        <v>518</v>
-      </c>
       <c r="H127" s="12" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I127" s="13" t="s">
         <v>145</v>
@@ -6492,22 +6492,22 @@
         <v>126</v>
       </c>
       <c r="C128" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D128" s="9" t="s">
+        <v>517</v>
+      </c>
+      <c r="E128" s="10" t="s">
+        <v>518</v>
+      </c>
+      <c r="F128" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="G128" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="E128" s="10" t="s">
+      <c r="H128" s="9" t="s">
         <v>520</v>
-      </c>
-      <c r="F128" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="G128" s="10" t="s">
-        <v>521</v>
-      </c>
-      <c r="H128" s="9" t="s">
-        <v>522</v>
       </c>
       <c r="I128" s="13" t="s">
         <v>145</v>
@@ -6524,22 +6524,22 @@
         <v>127</v>
       </c>
       <c r="C129" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D129" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="E129" s="13" t="s">
+        <v>522</v>
+      </c>
+      <c r="F129" s="12" t="s">
         <v>523</v>
       </c>
-      <c r="E129" s="13" t="s">
+      <c r="G129" s="13" t="s">
         <v>524</v>
       </c>
-      <c r="F129" s="12" t="s">
-        <v>525</v>
-      </c>
-      <c r="G129" s="13" t="s">
-        <v>526</v>
-      </c>
       <c r="H129" s="12" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I129" s="13" t="s">
         <v>145</v>
@@ -6556,22 +6556,22 @@
         <v>128</v>
       </c>
       <c r="C130" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D130" s="9" t="s">
+        <v>525</v>
+      </c>
+      <c r="E130" s="10" t="s">
+        <v>526</v>
+      </c>
+      <c r="F130" s="9" t="s">
         <v>527</v>
       </c>
-      <c r="E130" s="10" t="s">
+      <c r="G130" s="10" t="s">
         <v>528</v>
       </c>
-      <c r="F130" s="9" t="s">
+      <c r="H130" s="9" t="s">
         <v>529</v>
-      </c>
-      <c r="G130" s="10" t="s">
-        <v>530</v>
-      </c>
-      <c r="H130" s="9" t="s">
-        <v>531</v>
       </c>
       <c r="I130" s="13" t="s">
         <v>145</v>
@@ -6588,22 +6588,22 @@
         <v>129</v>
       </c>
       <c r="C131" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D131" s="12" t="s">
+        <v>530</v>
+      </c>
+      <c r="E131" s="13" t="s">
+        <v>531</v>
+      </c>
+      <c r="F131" s="12" t="s">
         <v>532</v>
       </c>
-      <c r="E131" s="13" t="s">
+      <c r="G131" s="13" t="s">
         <v>533</v>
       </c>
-      <c r="F131" s="12" t="s">
-        <v>534</v>
-      </c>
-      <c r="G131" s="13" t="s">
-        <v>535</v>
-      </c>
       <c r="H131" s="12" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I131" s="13" t="s">
         <v>145</v>
@@ -6620,22 +6620,22 @@
         <v>130</v>
       </c>
       <c r="C132" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D132" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="E132" s="10" t="s">
+        <v>535</v>
+      </c>
+      <c r="F132" s="9" t="s">
         <v>536</v>
       </c>
-      <c r="E132" s="10" t="s">
+      <c r="G132" s="10" t="s">
         <v>537</v>
       </c>
-      <c r="F132" s="9" t="s">
-        <v>538</v>
-      </c>
-      <c r="G132" s="10" t="s">
-        <v>539</v>
-      </c>
       <c r="H132" s="9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I132" s="13" t="s">
         <v>145</v>
@@ -6652,22 +6652,22 @@
         <v>131</v>
       </c>
       <c r="C133" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D133" s="12" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="E133" s="13" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="F133" s="9" t="s">
         <v>34</v>
       </c>
       <c r="G133" s="13" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="H133" s="12" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="I133" s="13" t="s">
         <v>145</v>
@@ -6684,22 +6684,22 @@
         <v>132</v>
       </c>
       <c r="C134" s="8" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D134" s="9" t="s">
+        <v>542</v>
+      </c>
+      <c r="E134" s="10" t="s">
+        <v>543</v>
+      </c>
+      <c r="F134" s="9" t="s">
         <v>544</v>
       </c>
-      <c r="E134" s="10" t="s">
+      <c r="G134" s="10" t="s">
         <v>545</v>
       </c>
-      <c r="F134" s="9" t="s">
-        <v>546</v>
-      </c>
-      <c r="G134" s="10" t="s">
-        <v>547</v>
-      </c>
       <c r="H134" s="9" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="I134" s="13" t="s">
         <v>145</v>
@@ -6719,19 +6719,19 @@
         <v>139</v>
       </c>
       <c r="D135" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="E135" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="F135" s="9" t="s">
         <v>548</v>
       </c>
-      <c r="E135" s="10" t="s">
+      <c r="G135" s="10" t="s">
         <v>549</v>
       </c>
-      <c r="F135" s="9" t="s">
+      <c r="H135" s="9" t="s">
         <v>550</v>
-      </c>
-      <c r="G135" s="10" t="s">
-        <v>551</v>
-      </c>
-      <c r="H135" s="9" t="s">
-        <v>552</v>
       </c>
       <c r="I135" s="13" t="s">
         <v>145</v>
@@ -6748,22 +6748,22 @@
         <v>134</v>
       </c>
       <c r="C136" s="11" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="D136" s="12" t="s">
+        <v>551</v>
+      </c>
+      <c r="E136" s="13" t="s">
+        <v>552</v>
+      </c>
+      <c r="F136" s="12" t="s">
+        <v>492</v>
+      </c>
+      <c r="G136" s="13" t="s">
         <v>553</v>
       </c>
-      <c r="E136" s="13" t="s">
+      <c r="H136" s="12" t="s">
         <v>554</v>
-      </c>
-      <c r="F136" s="12" t="s">
-        <v>494</v>
-      </c>
-      <c r="G136" s="13" t="s">
-        <v>555</v>
-      </c>
-      <c r="H136" s="12" t="s">
-        <v>556</v>
       </c>
       <c r="I136" s="13" t="s">
         <v>145</v>
@@ -6780,25 +6780,25 @@
         <v>135</v>
       </c>
       <c r="C137" s="8" t="s">
+        <v>555</v>
+      </c>
+      <c r="D137" s="9" t="s">
+        <v>556</v>
+      </c>
+      <c r="E137" s="10" t="s">
         <v>557</v>
       </c>
-      <c r="D137" s="9" t="s">
+      <c r="F137" s="9" t="s">
         <v>558</v>
       </c>
-      <c r="E137" s="10" t="s">
+      <c r="G137" s="10" t="s">
         <v>559</v>
       </c>
-      <c r="F137" s="9" t="s">
+      <c r="H137" s="9" t="s">
         <v>560</v>
       </c>
-      <c r="G137" s="10" t="s">
+      <c r="I137" s="10" t="s">
         <v>561</v>
-      </c>
-      <c r="H137" s="9" t="s">
-        <v>562</v>
-      </c>
-      <c r="I137" s="10" t="s">
-        <v>563</v>
       </c>
       <c r="J137" s="9">
         <v>1</v>
@@ -6812,25 +6812,25 @@
         <v>136</v>
       </c>
       <c r="C138" s="11" t="s">
+        <v>562</v>
+      </c>
+      <c r="D138" s="12" t="s">
+        <v>563</v>
+      </c>
+      <c r="E138" s="13" t="s">
         <v>564</v>
       </c>
-      <c r="D138" s="12" t="s">
+      <c r="F138" s="12" t="s">
         <v>565</v>
       </c>
-      <c r="E138" s="13" t="s">
+      <c r="G138" s="13" t="s">
         <v>566</v>
       </c>
-      <c r="F138" s="12" t="s">
+      <c r="H138" s="12" t="s">
         <v>567</v>
       </c>
-      <c r="G138" s="13" t="s">
+      <c r="I138" s="13" t="s">
         <v>568</v>
-      </c>
-      <c r="H138" s="12" t="s">
-        <v>569</v>
-      </c>
-      <c r="I138" s="13" t="s">
-        <v>570</v>
       </c>
       <c r="J138" s="12">
         <v>2</v>
@@ -6844,25 +6844,25 @@
         <v>137</v>
       </c>
       <c r="C139" s="8" t="s">
+        <v>569</v>
+      </c>
+      <c r="D139" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="E139" s="10" t="s">
         <v>571</v>
       </c>
-      <c r="D139" s="9" t="s">
+      <c r="F139" s="9" t="s">
         <v>572</v>
       </c>
-      <c r="E139" s="10" t="s">
+      <c r="G139" s="10" t="s">
         <v>573</v>
       </c>
-      <c r="F139" s="9" t="s">
+      <c r="H139" s="9" t="s">
         <v>574</v>
       </c>
-      <c r="G139" s="10" t="s">
-        <v>575</v>
-      </c>
-      <c r="H139" s="9" t="s">
-        <v>576</v>
-      </c>
       <c r="I139" s="10" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="J139" s="9">
         <v>1</v>
@@ -6875,22 +6875,22 @@
         <v>138</v>
       </c>
       <c r="C140" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D140" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E140" s="21" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="F140" s="18" t="s">
         <v>34</v>
       </c>
       <c r="G140" s="21" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H140" s="18" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="I140" s="21" t="s">
         <v>145</v>
@@ -6906,22 +6906,22 @@
         <v>139</v>
       </c>
       <c r="C141" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D141" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E141" s="21" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="F141" s="22" t="s">
         <v>34</v>
       </c>
       <c r="G141" s="21" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="H141" s="18" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="I141" s="21" t="s">
         <v>145</v>
@@ -6930,7 +6930,7 @@
         <v>1</v>
       </c>
       <c r="K141" s="23" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="36">
@@ -6939,22 +6939,22 @@
         <v>140</v>
       </c>
       <c r="C142" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D142" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E142" s="17" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="F142" s="22" t="s">
         <v>34</v>
       </c>
       <c r="G142" s="17" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="H142" s="22" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="I142" s="17" t="s">
         <v>145</v>
@@ -6970,22 +6970,22 @@
         <v>141</v>
       </c>
       <c r="C143" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D143" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E143" s="17" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="F143" s="22" t="s">
         <v>34</v>
       </c>
       <c r="G143" s="17" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="H143" s="22" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="I143" s="17" t="s">
         <v>145</v>
@@ -7001,13 +7001,13 @@
         <v>142</v>
       </c>
       <c r="C144" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D144" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E144" s="13" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="F144" s="22" t="s">
         <v>34</v>
@@ -7021,7 +7021,7 @@
         <v>1</v>
       </c>
       <c r="K144" s="9" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
     </row>
     <row r="145" spans="2:11" ht="24.75" thickBot="1">
@@ -7030,22 +7030,22 @@
         <v>143</v>
       </c>
       <c r="C145" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D145" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E145" s="17" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="F145" s="22" t="s">
         <v>34</v>
       </c>
       <c r="G145" s="17" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="H145" s="22" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="I145" s="17" t="s">
         <v>145</v>
@@ -7054,7 +7054,7 @@
         <v>1</v>
       </c>
       <c r="K145" s="22" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
     </row>
     <row r="146" spans="2:11" ht="24.75" thickBot="1">
@@ -7063,13 +7063,13 @@
         <v>144</v>
       </c>
       <c r="C146" s="20" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="D146" s="18" t="s">
         <v>145</v>
       </c>
       <c r="E146" s="13" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="F146" s="22" t="s">
         <v>34</v>
@@ -7078,7 +7078,7 @@
         <v>8900</v>
       </c>
       <c r="H146" s="22" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="I146" s="17" t="s">
         <v>145</v>

</xml_diff>